<commit_message>
Updated excel_template + added relative filepaths
</commit_message>
<xml_diff>
--- a/excel_template.xlsx
+++ b/excel_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pauls\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pauls\Documents\HES-battery-algo\Battery-algo\battery-optimizer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74EAF066-BD1D-43FE-BD0E-F0557AC0F8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9674721-BDE2-47A1-95C6-6850BEA7DDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabula" sheetId="1" r:id="rId1"/>
@@ -462,17 +462,6 @@
             <c:idx val="0"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000001-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -483,17 +472,6 @@
             <c:idx val="1"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -504,17 +482,6 @@
             <c:idx val="2"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000005-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -525,17 +492,6 @@
             <c:idx val="3"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000007-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -546,17 +502,6 @@
             <c:idx val="4"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000009-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -567,17 +512,6 @@
             <c:idx val="5"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000000B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -588,17 +522,6 @@
             <c:idx val="6"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000000D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -609,17 +532,6 @@
             <c:idx val="7"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000000F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -630,17 +542,6 @@
             <c:idx val="8"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000011-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -651,17 +552,6 @@
             <c:idx val="9"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000013-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -672,17 +562,6 @@
             <c:idx val="10"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000015-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -693,17 +572,6 @@
             <c:idx val="11"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000017-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -714,17 +582,6 @@
             <c:idx val="12"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000019-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -735,17 +592,6 @@
             <c:idx val="13"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000001B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -756,17 +602,6 @@
             <c:idx val="14"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000001D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -777,17 +612,6 @@
             <c:idx val="15"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000001F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -798,17 +622,6 @@
             <c:idx val="16"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000021-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -819,17 +632,6 @@
             <c:idx val="17"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000023-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -840,17 +642,6 @@
             <c:idx val="18"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000025-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -861,17 +652,6 @@
             <c:idx val="19"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000027-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -882,17 +662,6 @@
             <c:idx val="20"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000029-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -903,17 +672,6 @@
             <c:idx val="21"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000002B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -924,17 +682,6 @@
             <c:idx val="22"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000002D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -945,17 +692,6 @@
             <c:idx val="23"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000002F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -966,17 +702,6 @@
             <c:idx val="24"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000031-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -987,17 +712,6 @@
             <c:idx val="25"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000033-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1008,17 +722,6 @@
             <c:idx val="26"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000035-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1029,17 +732,6 @@
             <c:idx val="27"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000037-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1050,17 +742,6 @@
             <c:idx val="28"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000039-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1071,17 +752,6 @@
             <c:idx val="29"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000003B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1092,17 +762,6 @@
             <c:idx val="30"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000003D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1113,17 +772,6 @@
             <c:idx val="31"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000003F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1134,17 +782,6 @@
             <c:idx val="32"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000041-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1155,17 +792,6 @@
             <c:idx val="33"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000043-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1176,17 +802,6 @@
             <c:idx val="34"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000045-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1197,17 +812,6 @@
             <c:idx val="35"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000047-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1218,17 +822,6 @@
             <c:idx val="36"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000049-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1239,17 +832,6 @@
             <c:idx val="37"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000004B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1260,17 +842,6 @@
             <c:idx val="38"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000004D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1281,17 +852,6 @@
             <c:idx val="39"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000004F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1302,17 +862,6 @@
             <c:idx val="40"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000051-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1323,17 +872,6 @@
             <c:idx val="41"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000053-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1344,17 +882,6 @@
             <c:idx val="42"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000055-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1365,17 +892,6 @@
             <c:idx val="43"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000057-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1386,17 +902,6 @@
             <c:idx val="44"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000059-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1407,17 +912,6 @@
             <c:idx val="45"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000005B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1428,17 +922,6 @@
             <c:idx val="46"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000005D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1449,17 +932,6 @@
             <c:idx val="47"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000005F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1470,17 +942,6 @@
             <c:idx val="48"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000061-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1491,17 +952,6 @@
             <c:idx val="49"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000063-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1512,17 +962,6 @@
             <c:idx val="50"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000065-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1533,17 +972,6 @@
             <c:idx val="51"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000067-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1554,17 +982,6 @@
             <c:idx val="52"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000069-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1575,17 +992,6 @@
             <c:idx val="53"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000006B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1596,17 +1002,6 @@
             <c:idx val="54"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000006D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1617,17 +1012,6 @@
             <c:idx val="55"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000006F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1638,17 +1022,6 @@
             <c:idx val="56"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000071-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1659,17 +1032,6 @@
             <c:idx val="57"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000073-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1680,17 +1042,6 @@
             <c:idx val="58"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000075-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1701,17 +1052,6 @@
             <c:idx val="59"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000077-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1722,17 +1062,6 @@
             <c:idx val="60"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000079-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1743,17 +1072,6 @@
             <c:idx val="61"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000007B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1764,17 +1082,6 @@
             <c:idx val="62"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000007D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1785,17 +1092,6 @@
             <c:idx val="63"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000007F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1806,17 +1102,6 @@
             <c:idx val="64"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000081-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1827,17 +1112,6 @@
             <c:idx val="65"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000083-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1848,17 +1122,6 @@
             <c:idx val="66"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000085-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1869,17 +1132,6 @@
             <c:idx val="67"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000087-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1890,17 +1142,6 @@
             <c:idx val="68"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000089-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1911,17 +1152,6 @@
             <c:idx val="69"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000008B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1932,17 +1162,6 @@
             <c:idx val="70"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000008D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1953,17 +1172,6 @@
             <c:idx val="71"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000008F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1974,17 +1182,6 @@
             <c:idx val="72"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000091-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -1995,17 +1192,6 @@
             <c:idx val="73"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000093-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2016,17 +1202,6 @@
             <c:idx val="74"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000095-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2037,17 +1212,6 @@
             <c:idx val="75"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000097-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2058,17 +1222,6 @@
             <c:idx val="76"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000099-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2079,17 +1232,6 @@
             <c:idx val="77"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000009B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2100,17 +1242,6 @@
             <c:idx val="78"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000009D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2121,17 +1252,6 @@
             <c:idx val="79"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000009F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2142,17 +1262,6 @@
             <c:idx val="80"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000A1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2163,17 +1272,6 @@
             <c:idx val="81"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000A3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2184,17 +1282,6 @@
             <c:idx val="82"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000A5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2205,17 +1292,6 @@
             <c:idx val="83"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000A7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2226,17 +1302,6 @@
             <c:idx val="84"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000A9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2247,17 +1312,6 @@
             <c:idx val="85"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000AB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2268,17 +1322,6 @@
             <c:idx val="86"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000AD-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2289,17 +1332,6 @@
             <c:idx val="87"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000AF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2310,17 +1342,6 @@
             <c:idx val="88"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000B1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2331,17 +1352,6 @@
             <c:idx val="89"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000B3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2352,17 +1362,6 @@
             <c:idx val="90"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000B5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2373,17 +1372,6 @@
             <c:idx val="91"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000B7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2394,17 +1382,6 @@
             <c:idx val="92"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000B9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2415,17 +1392,6 @@
             <c:idx val="93"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000BB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2436,17 +1402,6 @@
             <c:idx val="94"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000BD-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2457,17 +1412,6 @@
             <c:idx val="95"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000BF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2478,17 +1422,6 @@
             <c:idx val="96"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000C1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2499,17 +1432,6 @@
             <c:idx val="97"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000C3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2520,17 +1442,6 @@
             <c:idx val="98"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000C5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2541,17 +1452,6 @@
             <c:idx val="99"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000C7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2562,17 +1462,6 @@
             <c:idx val="100"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000C9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2583,17 +1472,6 @@
             <c:idx val="101"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000CB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2604,17 +1482,6 @@
             <c:idx val="102"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000CD-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2625,17 +1492,6 @@
             <c:idx val="103"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000CF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2646,17 +1502,6 @@
             <c:idx val="104"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000D1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2667,17 +1512,6 @@
             <c:idx val="105"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000D3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2688,17 +1522,6 @@
             <c:idx val="106"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000D5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2709,17 +1532,6 @@
             <c:idx val="107"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000D7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2730,17 +1542,6 @@
             <c:idx val="108"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000D9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2751,17 +1552,6 @@
             <c:idx val="109"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000DB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2772,17 +1562,6 @@
             <c:idx val="110"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000DD-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2793,17 +1572,6 @@
             <c:idx val="111"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000DF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2814,17 +1582,6 @@
             <c:idx val="112"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000E1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2835,17 +1592,6 @@
             <c:idx val="113"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000E3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2856,17 +1602,6 @@
             <c:idx val="114"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000E5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2877,17 +1612,6 @@
             <c:idx val="115"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000E7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2898,17 +1622,6 @@
             <c:idx val="116"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000E9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2919,17 +1632,6 @@
             <c:idx val="117"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000EB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2940,17 +1642,6 @@
             <c:idx val="118"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000ED-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2961,17 +1652,6 @@
             <c:idx val="119"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000EF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -2982,17 +1662,6 @@
             <c:idx val="120"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000F1-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3003,17 +1672,6 @@
             <c:idx val="121"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000F3-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3024,17 +1682,6 @@
             <c:idx val="122"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000F5-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3045,17 +1692,6 @@
             <c:idx val="123"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000F7-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3066,17 +1702,6 @@
             <c:idx val="124"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000F9-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3087,17 +1712,6 @@
             <c:idx val="125"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000FB-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3108,17 +1722,6 @@
             <c:idx val="126"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000FD-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3129,17 +1732,6 @@
             <c:idx val="127"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{000000FF-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3150,17 +1742,6 @@
             <c:idx val="128"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000101-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3171,17 +1752,6 @@
             <c:idx val="129"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000103-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3192,17 +1762,6 @@
             <c:idx val="130"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000105-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3213,17 +1772,6 @@
             <c:idx val="131"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000107-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3234,17 +1782,6 @@
             <c:idx val="132"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000109-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3255,17 +1792,6 @@
             <c:idx val="133"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000010B-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3276,17 +1802,6 @@
             <c:idx val="134"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000010D-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3297,17 +1812,6 @@
             <c:idx val="135"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{0000010F-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3318,17 +1822,6 @@
             <c:idx val="136"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000111-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3339,17 +1832,6 @@
             <c:idx val="137"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000113-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3360,17 +1842,6 @@
             <c:idx val="138"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000115-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -3381,17 +1852,6 @@
             <c:idx val="139"/>
             <c:invertIfNegative val="1"/>
             <c:bubble3D val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000117-A1B3-42DF-9B3E-48BEECFB6895}"/>
@@ -8597,6 +7057,34 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:srgbClr val="FFFFFF"/>
+            </a:gs>
+            <a:gs pos="28571">
+              <a:srgbClr val="FFFFFF"/>
+            </a:gs>
+            <a:gs pos="28572">
+              <a:srgbClr val="E0E0E0"/>
+            </a:gs>
+            <a:gs pos="97143">
+              <a:srgbClr val="E0E0E0"/>
+            </a:gs>
+            <a:gs pos="97144">
+              <a:srgbClr val="FFFFFF"/>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:srgbClr val="FFFFFF"/>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="0"/>
+        </a:gradFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
@@ -8631,9 +7119,9 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.17564267270234951"/>
-          <c:y val="3.2784922997869032E-2"/>
-          <c:w val="0.33882989575695699"/>
+          <c:x val="2.187699733140052E-2"/>
+          <c:y val="1.5155128135917389E-2"/>
+          <c:w val="8.3599808915098994E-2"/>
           <c:h val="5.2667910730811798E-2"/>
         </c:manualLayout>
       </c:layout>
@@ -8705,14 +7193,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>298450</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>82550</xdr:rowOff>
     </xdr:to>
@@ -9040,7 +7528,7 @@
     <row r="1" spans="2:4" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="1">
         <f ca="1">TODAY()+1</f>
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3">

</xml_diff>